<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T17:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -830,6 +830,11 @@
           <t>13</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -837,6 +842,11 @@
           <t>130</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2, 3A, 3B1A, 3B1B1, 3B1B2, 3B1B3, 3B2, 3B3, 4A, 4B1, 4B2, 4B3, 5</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -844,6 +854,11 @@
           <t>131</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -851,6 +866,11 @@
           <t>132</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -858,6 +878,11 @@
           <t>133</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -865,6 +890,11 @@
           <t>134</t>
         </is>
       </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1A1, 1A1B, 1A2, 1A3A, 1A3B, 1B1, 1B2, 2, 3A1, 3A2, 3B1A, 3B1B, 3B1C, 3B1D, 3B1E, 3B2, 3B3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -872,6 +902,11 @@
           <t>135</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -879,6 +914,11 @@
           <t>136</t>
         </is>
       </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -886,6 +926,11 @@
           <t>137</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 2, 3A, 3B1, 3B2, 3B3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -893,6 +938,11 @@
           <t>138</t>
         </is>
       </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2A5, 2A6, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -900,6 +950,11 @@
           <t>139</t>
         </is>
       </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -907,6 +962,11 @@
           <t>14</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -914,6 +974,11 @@
           <t>140</t>
         </is>
       </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -921,6 +986,11 @@
           <t>141</t>
         </is>
       </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -928,6 +998,11 @@
           <t>142</t>
         </is>
       </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -935,6 +1010,11 @@
           <t>143</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -942,6 +1022,11 @@
           <t>144</t>
         </is>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -949,6 +1034,11 @@
           <t>145</t>
         </is>
       </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4A, 4B, 5, 6A, 6B, 7, 8A, 8B1, 8B2, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -956,6 +1046,11 @@
           <t>146</t>
         </is>
       </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -963,6 +1058,11 @@
           <t>147</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -970,6 +1070,11 @@
           <t>148</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -977,6 +1082,11 @@
           <t>149</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -984,6 +1094,11 @@
           <t>15</t>
         </is>
       </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -991,6 +1106,11 @@
           <t>150</t>
         </is>
       </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B, 7, 8A, 8B, 8C, 8D, 8E, 9</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -998,6 +1118,11 @@
           <t>151</t>
         </is>
       </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1005,6 +1130,11 @@
           <t>152</t>
         </is>
       </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1012,6 +1142,11 @@
           <t>153</t>
         </is>
       </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2B3, 3A1A, 3A1B, 3A1C, 3A1D, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1019,6 +1154,11 @@
           <t>154</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1026,6 +1166,11 @@
           <t>155</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B1, 3B2, 3C1, 3C2, 4, 5A, 5B, 5C, 5D, 5E1, 5E2</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1033,6 +1178,11 @@
           <t>156</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1040,6 +1190,11 @@
           <t>157</t>
         </is>
       </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>1, 10, 12, 13, 14, 2, 3, 4A, 4B, 4C, 4D, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1047,6 +1202,11 @@
           <t>158</t>
         </is>
       </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1054,6 +1214,11 @@
           <t>159</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 1D, 2A, 2B, 2C1, 2C2, 3A, 3B, 4A1, 4A2, 4B1, 4B2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1061,6 +1226,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1068,6 +1238,11 @@
           <t>160</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2B3, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1075,6 +1250,11 @@
           <t>161</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1082,6 +1262,11 @@
           <t>162</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1089,6 +1274,11 @@
           <t>163</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1096,6 +1286,11 @@
           <t>164</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1103,6 +1298,11 @@
           <t>165</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1110,6 +1310,11 @@
           <t>166</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1117,6 +1322,11 @@
           <t>167</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1124,6 +1334,11 @@
           <t>168</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 2A, 2B1, 2B2, 3A, 3B, 4, 5, 6, 7, 8, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1131,6 +1346,11 @@
           <t>169</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1138,6 +1358,11 @@
           <t>17</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10B, 11A, 11B, 11C, 2, 3, 4A1, 4A2, 4B1, 4B2, 4C, 4D, 4E, 5A, 5B, 6A1, 6A2, 6B, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1145,6 +1370,11 @@
           <t>170</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A1, 4A2, 4B, 5A1, 5A2, 5A3, 5B, 6A, 6B, 6C1, 6C2, 7A1, 7A2, 7B, 8A, 8B, 8C</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1152,6 +1382,11 @@
           <t>171</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1159,6 +1394,11 @@
           <t>172</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1166,6 +1406,11 @@
           <t>173</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1173,6 +1418,11 @@
           <t>174</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1180,6 +1430,11 @@
           <t>175</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2A1A, 2A2A1B, 2A2B, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1187,6 +1442,11 @@
           <t>176</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1194,6 +1454,11 @@
           <t>177</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1201,6 +1466,11 @@
           <t>178</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5, 1B, 2A, 2B1, 2B2, 2B3, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1208,6 +1478,11 @@
           <t>179</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1215,6 +1490,11 @@
           <t>18</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1222,6 +1502,11 @@
           <t>180</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1229,6 +1514,11 @@
           <t>181</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1236,6 +1526,11 @@
           <t>182</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1243,6 +1538,11 @@
           <t>183</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1250,6 +1550,11 @@
           <t>184</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1C, 1D1, 1D2, 2, 3A, 3C1, 3C2, 3D1, 3D2, 3E1, 3E2, 3F</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1257,6 +1562,11 @@
           <t>185</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1264,6 +1574,11 @@
           <t>186</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1, 1A2, 1B1A1, 1B2, 1B3, 1B4, 2A, 2B1, 2B1B, 2B2, 2C, 2C2, 2C3, 2C4, 2C5, 2C6, 3A1A, 3A1B, 3A1C, 3B, 3C, 3D, 3E, 4A, 4B, 4C, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1271,6 +1586,11 @@
           <t>187</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1278,6 +1598,11 @@
           <t>188</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 2A1A, 2A1B, 2A2, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1285,6 +1610,11 @@
           <t>189</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1292,6 +1622,11 @@
           <t>19</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1299,6 +1634,11 @@
           <t>190</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B, 3A, 3B, 4A1, 4A2, 4B, 4C, 5A, 5B, 5C, 5D, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1306,6 +1646,11 @@
           <t>191</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 2C, 2D1, 2D2, 2E, 3</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1313,6 +1658,11 @@
           <t>192</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1320,6 +1670,11 @@
           <t>193</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B1A, 2B2, 2B3, 2B4, 2B5, 3A1, 3A2, 3B1, 3B2, 3B3A1, 3B3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1327,6 +1682,11 @@
           <t>194</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1B1A1A1A1, 1B1B, 1B1C, 1B2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A1A1, 2A1B1, 2A1B2, 2A2, 2A3, 2B, 2C, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1334,6 +1694,11 @@
           <t>195</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 20, 21, 2A1A, 2A2, 2A3, 2B1A1, 2C1, 2C2, 3, 4A, 4B1, 4B2, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1341,6 +1706,11 @@
           <t>196</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A, 2A1B, 2A2A, 2A2B, 2A2C, 2B1, 2B2, 2B3, 2B4, 2C1A, 2C1B, 2C1C, 2C2A, 2C2B</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1348,6 +1718,11 @@
           <t>197</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1A1, 2A1B, 2A1C, 2A2, 2B1, 2B2, 2B3, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1355,6 +1730,11 @@
           <t>198</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 1C, 1D1, 1D2, 2A, 2B1, 2C, 3A1A, 3A2, 3B, 4A1A, 4A1B, 4B, 5A1, 5A2, 5B, 6, 7A1, 7A2, 7B, 8A1A1, 8A1A2, 8A1B, 8A2, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1362,6 +1742,11 @@
           <t>199</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1369,6 +1754,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1376,6 +1766,11 @@
           <t>200</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A1, 4A2, 4A3, 4B, 5A1, 5A2, 5B1, 5B2, 5C</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1383,6 +1778,11 @@
           <t>201</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1390,6 +1790,11 @@
           <t>202</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1397,6 +1802,11 @@
           <t>203</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1404,6 +1814,11 @@
           <t>204</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1411,6 +1826,11 @@
           <t>205</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1418,6 +1838,11 @@
           <t>206</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11A3, 11B, 11C, 12, 13, 14A1, 14A2, 14B, 14C, 15, 16A1A, 16A2, 16B, 17A1A, 17A2, 17B, 18, 19, 2, 20, 21, 23, 24, 3, 4, 5A, 5B, 5C, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1425,11 +1850,21 @@
           <t>207</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 3, 4, 5A1, 5A2, 5A3A, 5A3B, 5B, 6A, 6B, 7</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
           <t>208A</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 3A1A, 3A2, 3B1, 3B2, 3B3A, 3B3B, 3B4, 3B5, 4A1, 4A2, 4A3, 4A4, 4A5, 4B1, 4B2A, 4B2B, 4B2C, 4B2D, 4B2E, 4C1, 4C2, 4C3, 4C4, 4C5, 5A, 5B, 6, 7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T17:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -1874,6 +1874,11 @@
           <t>208B</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1881,6 +1886,11 @@
           <t>209</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1888,6 +1898,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1895,6 +1910,11 @@
           <t>210</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5, 6, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1902,6 +1922,11 @@
           <t>211A</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1909,6 +1934,11 @@
           <t>211B</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A1, 3A2, 3A3A, 3A3B, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1916,6 +1946,11 @@
           <t>212</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1923,11 +1958,21 @@
           <t>213A</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1A1A1A, 1A1A2, 1A1B, 1A2, 1B, 1C, 1D, 1E1, 1E2, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
           <t>213B</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T17:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -1982,6 +1982,11 @@
           <t>214A</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1989,6 +1994,11 @@
           <t>214B</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1996,6 +2006,11 @@
           <t>215</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C1A, 1C2, 1C3, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2003,6 +2018,11 @@
           <t>216</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2010,6 +2030,11 @@
           <t>217A</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2, 1B1, 1B2, 1C, 2A1, 2A2, 2B1, 2B2A, 2B2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2017,6 +2042,11 @@
           <t>217B</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 2A1A, 2A1B, 2A1C, 2A1D1, 2A1D2, 2A1E1, 2A1E2, 2A1H, 2A2A1, 2A2A2, 2A2B1, 2A2B2, 2B1, 2B2A, 2C1A, 2C1B, 2C1C1, 2C1C2, 2C1C3, 2C1C4, 2C1C5, 2C1C6, 2C2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2024,6 +2054,11 @@
           <t>218</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2031,6 +2066,11 @@
           <t>219</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 2, 3, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2038,6 +2078,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2045,6 +2090,11 @@
           <t>220</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2052,6 +2102,11 @@
           <t>221</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2059,6 +2114,11 @@
           <t>222</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2066,6 +2126,11 @@
           <t>224</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 3C1, 3C2, 4A1A, 4B, 4C, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -2073,6 +2138,11 @@
           <t>225</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B1, 2B2, 2B3A, 2B3B, 3A1A, 3A1B, 3A2, 3B1, 3B2, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -2080,6 +2150,11 @@
           <t>226</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -2087,6 +2162,11 @@
           <t>227</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1A, 2B1B, 2B1C, 2B2, 2B3, 2B4, 2B5, 3A1, 3A2, 3B1, 3B2, 3C1, 3C2</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -2094,6 +2174,11 @@
           <t>228</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2101,6 +2186,11 @@
           <t>229</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5A1, 5A2, 5B, 5C, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2108,6 +2198,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2115,6 +2210,11 @@
           <t>230</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2122,6 +2222,11 @@
           <t>231</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D, 1E, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -2129,6 +2234,11 @@
           <t>232</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2136,6 +2246,11 @@
           <t>233</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5A, 5B, 5C1, 5C2</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -2143,6 +2258,11 @@
           <t>234</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2150,6 +2270,11 @@
           <t>235</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -2157,6 +2282,11 @@
           <t>236</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -2164,6 +2294,11 @@
           <t>237</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -2171,6 +2306,11 @@
           <t>238</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -2178,6 +2318,11 @@
           <t>239</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -2185,6 +2330,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -2192,6 +2342,11 @@
           <t>240</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3A, 3B, 3C1, 3C2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -2199,6 +2354,11 @@
           <t>241A</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 2A1, 2A2, 2A3, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -2206,6 +2366,11 @@
           <t>241B</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 2A, 2B1, 2B2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -2213,6 +2378,11 @@
           <t>242A</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2220,6 +2390,11 @@
           <t>242B</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1, 1B, 1C, 2A, 2A1A, 2B, 3, 4, 5, 6, 7, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2227,6 +2402,11 @@
           <t>243</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A1, 1B1A2, 1B1B, 1B2, 2, 3A, 3B, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2234,6 +2414,11 @@
           <t>244</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2241,6 +2426,11 @@
           <t>245</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2248,6 +2438,11 @@
           <t>246</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B1, 7B2, 7B3, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2255,6 +2450,11 @@
           <t>247</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2262,6 +2462,11 @@
           <t>248</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2269,6 +2474,11 @@
           <t>249</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2276,6 +2486,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 3C, 3D, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2283,6 +2498,11 @@
           <t>250</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2290,6 +2510,11 @@
           <t>251</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -2297,6 +2522,11 @@
           <t>252</t>
         </is>
       </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -2304,6 +2534,11 @@
           <t>253</t>
         </is>
       </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -2311,6 +2546,11 @@
           <t>254</t>
         </is>
       </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -2318,6 +2558,11 @@
           <t>255</t>
         </is>
       </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5, 1B1A, 1B1B, 1B2, 2A, 2B, 2C, 3A, 3B, 4, 5, 6A1, 6A2, 6A3, 6B1, 6B2, 6B3</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -2325,6 +2570,11 @@
           <t>256</t>
         </is>
       </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2, 1B, 1C, 2, 3A, 3B1A, 3B1B, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -2332,6 +2582,11 @@
           <t>257</t>
         </is>
       </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -2339,6 +2594,11 @@
           <t>258</t>
         </is>
       </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 1D, 1E, 1F, 1G, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -2346,6 +2606,11 @@
           <t>259</t>
         </is>
       </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -2353,6 +2618,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -2360,6 +2630,11 @@
           <t>260</t>
         </is>
       </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -2367,6 +2642,11 @@
           <t>261</t>
         </is>
       </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A2C, 1B, 1C1A, 1C1B, 1C2, 2A1A, 2A1B, 2A1C, 2A1D, 2A1E, 2A2, 2B, 3A, 3B, 4, 5A1A, 5A1B, 5A1C, 5A1D, 5A2, 5B1, 5B2, 5C, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -2374,6 +2654,11 @@
           <t>262</t>
         </is>
       </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -2381,6 +2666,11 @@
           <t>263</t>
         </is>
       </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -2388,6 +2678,11 @@
           <t>264</t>
         </is>
       </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D, 3A, 3B, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -2395,6 +2690,11 @@
           <t>265</t>
         </is>
       </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -2402,6 +2702,11 @@
           <t>266</t>
         </is>
       </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -2409,6 +2714,11 @@
           <t>267</t>
         </is>
       </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -2416,6 +2726,11 @@
           <t>268</t>
         </is>
       </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -2423,6 +2738,11 @@
           <t>269</t>
         </is>
       </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -2430,6 +2750,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2A1, 2A2, 2B, 3A1, 3A2, 3A3, 3B1, 3B2, 3B3, 4A1, 4A2, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -2437,6 +2762,11 @@
           <t>270</t>
         </is>
       </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -2444,6 +2774,11 @@
           <t>271</t>
         </is>
       </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 2B3</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -2451,6 +2786,11 @@
           <t>272</t>
         </is>
       </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -2458,6 +2798,11 @@
           <t>273</t>
         </is>
       </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -2465,6 +2810,11 @@
           <t>274</t>
         </is>
       </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B, 1B2, 1C, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -2472,6 +2822,11 @@
           <t>275</t>
         </is>
       </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -2479,6 +2834,11 @@
           <t>276</t>
         </is>
       </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 2A1, 2B, 2C, 2D, 2E, 2F, 2G, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -2486,6 +2846,11 @@
           <t>277</t>
         </is>
       </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -2493,6 +2858,11 @@
           <t>278</t>
         </is>
       </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -2500,6 +2870,11 @@
           <t>279</t>
         </is>
       </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -2507,6 +2882,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -2514,6 +2894,11 @@
           <t>280</t>
         </is>
       </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 1A, 1B, 2, 3A, 3B, 3C1, 3C2, 3C3, 3C4, 4A, 4B, 5, 6, 7A, 7B, 8A1, 8A2, 8B, 9A, 9B, 9C, 9D</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -2521,6 +2906,11 @@
           <t>281</t>
         </is>
       </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -2528,6 +2918,11 @@
           <t>282</t>
         </is>
       </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -2535,6 +2930,11 @@
           <t>283</t>
         </is>
       </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -2542,6 +2942,11 @@
           <t>284</t>
         </is>
       </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -2549,6 +2954,11 @@
           <t>285</t>
         </is>
       </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3A, 2A3B, 2A3C, 2B, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -2556,6 +2966,11 @@
           <t>286</t>
         </is>
       </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -2563,6 +2978,11 @@
           <t>287</t>
         </is>
       </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>1, 2, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -2570,11 +2990,21 @@
           <t>288</t>
         </is>
       </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
           <t>289</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>1, 2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T17:50:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -3014,6 +3014,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1C, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -3021,6 +3026,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -3028,6 +3038,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B, 3A, 3B1, 3B2, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -3035,6 +3050,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -3042,6 +3062,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -3049,6 +3074,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -3056,6 +3086,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -3063,6 +3098,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -3070,6 +3110,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -3077,6 +3122,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -3084,6 +3134,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -3091,6 +3146,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -3098,6 +3158,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -3105,6 +3170,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -3112,6 +3182,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2B3, 3A, 3B, 3C, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -3119,6 +3194,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A1, 4A2, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -3126,6 +3206,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -3133,11 +3218,21 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
           <t>306</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 65 village workbooks (sivaramans-llin 2026-10-10T18:00:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -3242,6 +3242,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -3249,6 +3254,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -3256,6 +3266,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2A5, 2A6, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -3263,6 +3278,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -3270,6 +3290,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -3277,6 +3302,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -3284,6 +3314,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -3291,6 +3326,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -3298,6 +3338,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -3305,6 +3350,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -3312,6 +3362,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -3319,6 +3374,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -3326,6 +3386,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A2A, 1A2B, 1B1A, 1B1B, 1B1C, 1B1D, 1B2A, 1B2B, 1B2C, 1C1A, 1C1B, 1C1C, 1C2A, 1C2B, 1D, 1E, 1F, 1G, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -3333,6 +3398,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -3340,6 +3410,11 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -3347,6 +3422,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3A1, 3A2, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -3354,6 +3434,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -3361,6 +3446,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E1, 1E2, 2A1, 2A2, 2A3, 2A4, 2A5, 2A6, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -3368,6 +3458,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B1A, 1B1B, 1B2, 1B3, 2A1A, 2A2, 2B1A, 2B2, 2C1, 2C2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -3375,6 +3470,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A1A1A, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34A, 34B, 35, 36, 37A, 37B, 37C, 38, 39, 3A1A1A, 40, 41, 42, 43, 44, 45, 4A1A, 4B, 5B1A, 5B2, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -3382,6 +3482,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1A1, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -3389,6 +3494,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 1A, 1B1A, 1B1B, 1B2, 2A, 2A2, 2B, 3A, 3A1B, 3A2, 3A3, 3B, 3C, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -3396,6 +3506,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -3403,6 +3518,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1A2, 1A1B1, 1A1B2, 1A1C, 1A2, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -3410,6 +3530,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -3417,6 +3542,11 @@
           <t>33</t>
         </is>
       </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -3424,6 +3554,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -3431,6 +3566,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -3438,6 +3578,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B1, 2B2, 3A, 3B1, 3B2, 4</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -3445,6 +3590,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -3452,6 +3602,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -3459,6 +3614,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -3466,6 +3626,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -3473,6 +3638,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -3480,6 +3650,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -3487,6 +3662,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -3494,6 +3674,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -3501,6 +3686,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B1, 4B2, 4B3, 4B4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -3508,6 +3698,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -3515,6 +3710,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>1, 2, 2A1B1, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -3522,6 +3722,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>10, 100A, 100B, 100C, 101, 102, 103, 104, 105, 106, 107, 108, 109, 11, 110, 111, 112, 113, 114, 115, 116, 117, 118, 119, 12, 120, 121, 122, 123, 124, 125, 13, 14, 15, 16, 17, 18, 19, 1A1C1, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 3A1A, 40, 41, 42, 43, 44, 45, 46, 47, 49, 4B2, 50, 51, 52, 53, 54, 55, 56, 57, 58A, 58B, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 8, 80, 81, 82, 83, 84, 85, 86A, 86B, 87, 88A, 88B, 89, 9, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -3529,6 +3734,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A1, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -3536,6 +3746,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>1A1A1A1, 1A1A2, 1A1B1, 1A1B2, 1A2, 1A3, 1B3A1, 1B3A2, 1B3B, 2, 2A, 3A1A1, 3A2, 3A3, 3A4, 3A5, 3A6, 3A7, 3A8, 3A9, 3B, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -3543,6 +3758,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -3550,6 +3770,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>10, 11, 119, 12, 13, 14, 1A1A1A, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 2B, 38, 39, 3A1B, 3A1C, 3A1D, 3A1E, 3A2, 40, 41, 5, 6, 7, 8A1, 8A2, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -3557,6 +3782,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>10, 11, 13, 14, 15, 16, 17, 18, 19, 1A1A, 1A2, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42A1A, 42A1B, 42A2, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -3564,6 +3794,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 14, 15A, 15B, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 8</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3571,6 +3806,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2, 3B3, 4, 5A, 5B, 6A, 6B, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3578,6 +3818,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3585,6 +3830,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3592,6 +3842,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>1A1, 1A2A, 1A2B, 1B, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3599,6 +3854,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3606,6 +3866,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 4, 5A, 5B, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3613,6 +3878,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1, 1A1, 1A2, 2, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3620,6 +3890,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3627,6 +3902,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3A, 3B, 4A, 4B, 5A, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3634,6 +3914,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B, 1C, 1D, 2A, 2B, 2C, 2D, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3641,6 +3926,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2B, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3648,6 +3938,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3655,6 +3950,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A1, 13A2, 13B, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3662,6 +3962,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3669,6 +3974,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3676,6 +3986,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3683,6 +3998,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3690,6 +4010,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 5A, 5B, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3697,6 +4022,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3704,6 +4034,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3711,6 +4046,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1A, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3718,6 +4058,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 19A, 19B, 2, 20, 21, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3725,6 +4070,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3732,6 +4082,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B1, 2B2, 3A, 3B, 3C, 3D, 4, 5A1, 5A2, 5B, 6A, 6B1, 6B2, 7, 8A1, 8A2, 8B1, 8B2</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3739,6 +4094,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3746,6 +4106,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3753,6 +4118,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A1, 2A2, 2A3, 2B, 2C, 3A, 3B, 3C, 3D, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3760,11 +4130,21 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
           <t>45</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B1, 2B2, 3A, 3B, 3C, 3D, 4A, 4B, 4C, 5A, 5B, 6A, 6B, 7A1, 7A2, 7B1, 7B2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 66 village workbooks (sivaramans-llin 2026-10-10T18:10:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Valuthalamdedu_13.42741_80.158148.xlsx
@@ -4154,6 +4154,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4161,6 +4166,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2B, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4168,6 +4178,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B, 4C, 5A, 5B, 6A, 6B1, 6B2, 7</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4175,6 +4190,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A1, 5A2, 5B, 6, 7A, 7B, 7C, 8A1, 8A2, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4182,6 +4202,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4189,6 +4214,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B1, 3B2</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4196,6 +4226,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4203,6 +4238,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4210,6 +4250,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2, 3A1, 3A2, 3B, 4A, 4B, 5A, 5B, 6A1, 6A2A, 6A2B, 6A3, 6A4, 6A5, 6A6, 6A7, 6A8, 6B, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4217,6 +4262,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4224,6 +4274,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4231,6 +4286,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 2C1, 2C2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4238,6 +4298,11 @@
           <t>58</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4245,6 +4310,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4252,6 +4322,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4259,6 +4334,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4266,6 +4346,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 2D, 2E, 2F</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4273,6 +4358,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4280,6 +4370,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4287,6 +4382,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4294,6 +4394,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4301,6 +4406,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1B3A, 1B4, 1B5, 1B6A, 1B6B, 1B7, 2A1, 2A2, 2B, 2C, 2D, 2E, 2F1, 2F2, 2G, 2H, 3A, 3B, 3C, 4A1, 4A2, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4308,6 +4418,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1B3, 1B4, 2A, 2B1, 2B2, 2B3, 2B4, 2B5, 2B6, 2B7, 2B8A, 2B8B, 2B9</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4315,6 +4430,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1A1A, 1A2, 1A3, 1B, 1C, 2A1A, 2A1B, 2A1C, 2A2, 2B1, 2B2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4322,6 +4442,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1A, 1C1B, 1C2, 1D, 2A1, 2A2, 2B1A1, 2B1B, 2B2, 2B3, 3A, 3B, 3C, 3D, 3E, 3F, 3G, 4A1, 4A2, 4A3, 4A4, 4B, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4329,6 +4454,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2A, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4336,6 +4466,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A2, 1B1A, 1B1B, 1B2, 1C1, 1C2, 1D1, 1D2A1, 1D3A, 20, 21, 22, 23A, 23B, 24, 25, 26, 27, 28, 29, 2A1A, 2A1B, 2A2, 2B, 2C, 3, 30, 31, 32, 33, 4, 5A1, 5A2A1, 5A2B1A1, 5B, 5C, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4343,6 +4478,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4350,6 +4490,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4357,6 +4502,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 1A1, 1A2, 1B, 1C, 2A, 2B, 3A, 3B, 4A, 4B1, 4B2, 5A, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4364,6 +4514,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>10, 1A, 1B1, 1B2, 1C, 2A, 2B, 3A, 3B, 4, 5A, 5B, 5C, 6, 7A, 7B, 7C, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4371,6 +4526,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1C, 2A, 2B, 2C, 2D, 3A, 3B, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4378,6 +4538,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3A1, 3A2, 3A3A, 3A3B, 3B, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4385,6 +4550,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1, 12A2, 12B, 13, 2, 3, 4, 5, 6, 7A1, 7A2, 7A3, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4392,6 +4562,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4399,6 +4574,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -4406,6 +4586,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C1, 2C2, 2D</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -4413,6 +4598,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 2, 3A, 3B, 4, 5, 6, 7, 8, 9A, 9B, 9C1, 9C2</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -4420,6 +4610,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -4427,6 +4622,11 @@
           <t>82</t>
         </is>
       </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2C1, 2C2A1, 2C2B, 2D1, 2D2, 2E, 3A1, 3A2, 3B1, 3B2A, 3B2B, 3B3, 3B4, 3B5, 3B6, 3B7, 4</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -4434,6 +4634,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 2, 3, 4A, 4B, 4C, 5, 6A, 6B1, 6B2, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -4441,6 +4646,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -4448,6 +4658,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 1I, 1J, 1K, 2</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -4455,6 +4670,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3A1, 3A2, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -4462,6 +4682,11 @@
           <t>87</t>
         </is>
       </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -4469,6 +4694,11 @@
           <t>88</t>
         </is>
       </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -4476,6 +4706,11 @@
           <t>89</t>
         </is>
       </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -4483,6 +4718,11 @@
           <t>9</t>
         </is>
       </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -4490,6 +4730,11 @@
           <t>90</t>
         </is>
       </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A1, 4A2, 4B1, 4B2</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -4497,6 +4742,11 @@
           <t>91</t>
         </is>
       </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -4504,6 +4754,11 @@
           <t>92</t>
         </is>
       </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -4511,6 +4766,11 @@
           <t>93</t>
         </is>
       </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3</t>
+        </is>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -4518,6 +4778,11 @@
           <t>94</t>
         </is>
       </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -4525,6 +4790,11 @@
           <t>95</t>
         </is>
       </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -4532,6 +4802,11 @@
           <t>96</t>
         </is>
       </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -4539,6 +4814,11 @@
           <t>97</t>
         </is>
       </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -4546,11 +4826,21 @@
           <t>98</t>
         </is>
       </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
           <t>99</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>